<commit_message>
Regenerate example workbooks with gen-examples
No functional/source changes; these were regenerated locally while
testing scripts/package-release.ps1 for the v1.0.0 release and reflect
the current gen-examples output. Not a release (no version bump/tag).

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/examples/07-inspecting-results.xlsx
+++ b/docs/examples/07-inspecting-results.xlsx
@@ -1,34 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Home\Github\cvxx\docs\examples\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50DA79FA-03D7-4E7C-A114-76AF54193B34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Inspecting Results" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -260,8 +241,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -372,8 +353,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -384,34 +368,19 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -449,7 +418,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -483,7 +452,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -518,10 +486,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -694,490 +661,490 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F44"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="34.7265625" customWidth="1"/>
-    <col min="2" max="5" width="18.7265625" customWidth="1"/>
-    <col min="6" max="6" width="58.7265625" customWidth="1"/>
+    <col min="1" max="1" width="34.7109375" customWidth="1"/>
+    <col min="2" max="5" width="18.7109375" customWidth="1"/>
+    <col min="6" max="6" width="58.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-    </row>
-    <row r="2" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="8" t="s">
+    <row r="1" spans="1:6" ht="30" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:6" ht="33.75" customHeight="1">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-    </row>
-    <row r="3" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="8" t="s">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" spans="1:6" ht="33.75" customHeight="1">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="2" t="s">
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:6">
+      <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="5">
         <v>2.5</v>
       </c>
-      <c r="F6" s="1"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
+      <c r="F6" s="2"/>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="5">
         <v>1.8</v>
       </c>
-      <c r="F7" s="1"/>
-    </row>
-    <row r="8" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="5">
         <v>24</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:6">
+      <c r="A10" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="2" t="s">
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
+    <row r="11" spans="1:6">
+      <c r="A11" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="5" t="str">
-        <f>_xll.CVX.VARIABLE(1,1,"qty_bread")</f>
-        <v>cvx:var:fdafe7c9-679e-4d85-a7c6-3f8dde112820</v>
-      </c>
-      <c r="F11" s="1" t="s">
+      <c r="B11" s="6">
+        <f>CVX.VARIABLE(1,1,"qty_bread")</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
+    <row r="12" spans="1:6">
+      <c r="A12" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="5" t="str">
-        <f>_xll.CVX.VARIABLE(1,1,"qty_milk")</f>
-        <v>cvx:var:9a8669c1-32c2-400f-99ec-3850dbcf9f85</v>
-      </c>
-      <c r="F12" s="1" t="s">
+      <c r="B12" s="6">
+        <f>CVX.VARIABLE(1,1,"qty_milk")</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
+    <row r="13" spans="1:6">
+      <c r="A13" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="5" t="str">
-        <f>_xll.CVX.EXPRESSION("2.5 * qty_bread + 1.8 * qty_milk","weekly_cost")</f>
-        <v>cvx:expr:bccf6f22-a769-4e88-a28a-ec3a8d651f19</v>
-      </c>
-      <c r="F13" s="1" t="s">
+      <c r="B13" s="6">
+        <f>CVX.EXPRESSION("2.5 * qty_bread + 1.8 * qty_milk","weekly_cost")</f>
+        <v>0</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A14" s="3" t="s">
+    <row r="14" spans="1:6">
+      <c r="A14" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="5" t="str">
-        <f>_xll.CVX.CONSTRAINT("6 * qty_bread + 8 * qty_milk &gt;= 24","protein_requirement")</f>
-        <v>cvx:constr:e3df6abe-b319-4510-98f5-318137360a10</v>
-      </c>
-      <c r="F14" s="1" t="s">
+      <c r="B14" s="6">
+        <f>CVX.CONSTRAINT("6 * qty_bread + 8 * qty_milk &gt;= 24","protein_requirement")</f>
+        <v>0</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
+    <row r="15" spans="1:6">
+      <c r="A15" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="5" t="str">
-        <f>_xll.CVX.CONSTRAINT("120 * qty_bread + 150 * qty_milk &gt;= 600","calorie_requirement")</f>
-        <v>cvx:constr:78e573fa-df85-4eb6-8b14-a2015f106058</v>
-      </c>
-      <c r="F15" s="1" t="s">
+      <c r="B15" s="6">
+        <f>CVX.CONSTRAINT("120 * qty_bread + 150 * qty_milk &gt;= 600","calorie_requirement")</f>
+        <v>0</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" s="3" t="s">
+    <row r="16" spans="1:6">
+      <c r="A16" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="5" t="str">
-        <f>_xll.CVX.CONSTRAINT("qty_bread &gt;= 0","bread_nonneg")</f>
-        <v>cvx:constr:05d5830d-7b8a-41fa-817b-e850c3b05d70</v>
-      </c>
-      <c r="F16" s="1" t="s">
+      <c r="B16" s="6">
+        <f>CVX.CONSTRAINT("qty_bread &gt;= 0","bread_nonneg")</f>
+        <v>0</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" s="3" t="s">
+    <row r="17" spans="1:6">
+      <c r="A17" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="5" t="str">
-        <f>_xll.CVX.CONSTRAINT("qty_milk &gt;= 0","milk_nonneg")</f>
-        <v>cvx:constr:bff7e919-59ac-447f-9f44-a280261e7940</v>
-      </c>
-      <c r="F17" s="1" t="s">
+      <c r="B17" s="6">
+        <f>CVX.CONSTRAINT("qty_milk &gt;= 0","milk_nonneg")</f>
+        <v>0</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A18" s="3" t="s">
+    <row r="18" spans="1:6">
+      <c r="A18" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="5" t="str">
-        <f>_xll.CVX.CONSTRAINTS(B14:B17,"diet_constraints")</f>
-        <v>cvx:constrset:d2a9b6a5-29c0-431a-9fe8-bab44097a4b2</v>
-      </c>
-      <c r="F18" s="1" t="s">
+      <c r="B18" s="6">
+        <f>CVX.CONSTRAINTS(B14:B17,"diet_constraints")</f>
+        <v>0</v>
+      </c>
+      <c r="F18" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="3" t="s">
+    <row r="19" spans="1:6">
+      <c r="A19" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="5" t="str">
-        <f>_xll.CVX.MINIMIZE(B13,"minimize_cost")</f>
-        <v>cvx:obj:efb5f2e8-2647-40b1-a7cc-f3a257ba32e5</v>
-      </c>
-      <c r="F19" s="1" t="s">
+      <c r="B19" s="6">
+        <f>CVX.MINIMIZE(B13,"minimize_cost")</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A20" s="3" t="s">
+    <row r="20" spans="1:6">
+      <c r="A20" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="5" t="str">
-        <f>_xll.CVX.PROBLEM(B19,B18,"diet_problem")</f>
-        <v>cvx:prob:75bc854a-7e7c-4eb6-8f0a-313876bc9962</v>
-      </c>
-      <c r="F20" s="1" t="s">
+      <c r="B20" s="6">
+        <f>CVX.PROBLEM(B19,B18,"diet_problem")</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" s="3" t="s">
+    <row r="21" spans="1:6">
+      <c r="A21" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="5" t="str">
-        <f>_xll.CVX.SOLVE(B20,"diet_result")</f>
-        <v>cvx:result:815426d7-ae99-405e-a662-2016a93c6cd0</v>
-      </c>
-      <c r="F21" s="1" t="s">
+      <c r="B21" s="6">
+        <f>CVX.SOLVE(B20,"diet_result")</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" s="2" t="s">
+    <row r="23" spans="1:6">
+      <c r="A23" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="2" t="s">
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" s="3" t="s">
+    <row r="24" spans="1:6">
+      <c r="A24" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B24" s="5" t="str">
-        <f>_xll.CVX.STATUS(B21)</f>
-        <v>optimal</v>
-      </c>
-      <c r="F24" s="1" t="s">
+      <c r="B24" s="6">
+        <f>CVX.STATUS(B21)</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="3" t="s">
+    <row r="25" spans="1:6">
+      <c r="A25" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="5">
-        <f>_xll.CVX.OBJECTIVE_VALUE(B21)</f>
-        <v>7.2000000005165168</v>
-      </c>
-      <c r="F25" s="1" t="s">
+      <c r="B25" s="6">
+        <f>CVX.OBJECTIVE_VALUE(B21)</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A26" s="3" t="s">
+    <row r="26" spans="1:6">
+      <c r="A26" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B26" s="5">
-        <f>_xll.CVX.VALUE(B21,B11)</f>
-        <v>1.3085414715514723E-10</v>
-      </c>
-      <c r="F26" s="1" t="s">
+      <c r="B26" s="6">
+        <f>CVX.VALUE(B21,B11)</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A27" s="3" t="s">
+    <row r="27" spans="1:6">
+      <c r="A27" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B27" s="5">
-        <f>_xll.CVX.VALUE(B21,B12)</f>
-        <v>4.0000000001052118</v>
-      </c>
-      <c r="F27" s="1" t="s">
+      <c r="B27" s="6">
+        <f>CVX.VALUE(B21,B12)</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A29" s="2" t="s">
+    <row r="29" spans="1:6">
+      <c r="A29" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B29" s="9" t="s">
+      <c r="B29" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="9"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
-      <c r="F29" s="2" t="s">
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A30" s="3" t="s">
+    <row r="30" spans="1:6">
+      <c r="A30" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B30" s="5" t="str">
-        <f>_xll.CVX.TYPE(B11)</f>
-        <v>variable</v>
-      </c>
-      <c r="F30" s="1" t="s">
+      <c r="B30" s="6">
+        <f>CVX.TYPE(B11)</f>
+        <v>0</v>
+      </c>
+      <c r="F30" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A31" s="3" t="s">
+    <row r="31" spans="1:6">
+      <c r="A31" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B31" s="5" t="str">
-        <f>_xll.CVX.TYPE(B19)</f>
-        <v>objective</v>
-      </c>
-      <c r="F31" s="1" t="s">
+      <c r="B31" s="6">
+        <f>CVX.TYPE(B19)</f>
+        <v>0</v>
+      </c>
+      <c r="F31" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A32" s="3" t="s">
+    <row r="32" spans="1:6">
+      <c r="A32" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B32" s="5" t="str">
-        <f>_xll.CVX.TYPE(B20)</f>
-        <v>problem</v>
-      </c>
-      <c r="F32" s="1" t="s">
+      <c r="B32" s="6">
+        <f>CVX.TYPE(B20)</f>
+        <v>0</v>
+      </c>
+      <c r="F32" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A33" s="3" t="s">
+    <row r="33" spans="1:6">
+      <c r="A33" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B33" s="5" t="str">
-        <f>_xll.CVX.TYPE(B21)</f>
-        <v>result</v>
-      </c>
-      <c r="F33" s="1" t="s">
+      <c r="B33" s="6">
+        <f>CVX.TYPE(B21)</f>
+        <v>0</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A34" s="3" t="s">
+    <row r="34" spans="1:6">
+      <c r="A34" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B34" s="5" t="str">
-        <f>_xll.CVX.SHAPE(B11)</f>
-        <v>1x1</v>
-      </c>
-      <c r="F34" s="1" t="s">
+      <c r="B34" s="6">
+        <f>CVX.SHAPE(B11)</f>
+        <v>0</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A35" s="3" t="s">
+    <row r="35" spans="1:6">
+      <c r="A35" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B35" s="5" t="str">
-        <f>_xll.CVX.DESCRIBE(B20)</f>
-        <v>"diet_problem" (cvx:prob:75bc854a-7e7c-4eb6-8f0a-313876bc9962): problem: objective="minimize_cost", constraints=[4]: "protein_requirement", "calorie_requirement", "bread_nonneg", "milk_nonneg", variables=[2]: "qty_bread", "qty_milk"</v>
-      </c>
-      <c r="F35" s="1" t="s">
+      <c r="B35" s="6">
+        <f>CVX.DESCRIBE(B20)</f>
+        <v>0</v>
+      </c>
+      <c r="F35" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A37" s="2" t="s">
+    <row r="37" spans="1:6">
+      <c r="A37" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="B37" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="2" t="s">
+      <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A38" s="3" t="s">
+    <row r="38" spans="1:6">
+      <c r="A38" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B38" s="6" t="str">
-        <f>_xll.CVX.STATUS(B21)</f>
-        <v>optimal</v>
-      </c>
-      <c r="F38" s="1" t="s">
+      <c r="B38" s="7">
+        <f>CVX.STATUS(B21)</f>
+        <v>0</v>
+      </c>
+      <c r="F38" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A39" s="3" t="s">
+    <row r="39" spans="1:6">
+      <c r="A39" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B39" s="6">
-        <f>_xll.CVX.OBJECTIVE_VALUE(B21)</f>
-        <v>7.2000000005165168</v>
-      </c>
-      <c r="F39" s="1" t="s">
+      <c r="B39" s="7">
+        <f>CVX.OBJECTIVE_VALUE(B21)</f>
+        <v>0</v>
+      </c>
+      <c r="F39" s="2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A40" s="3" t="s">
+    <row r="40" spans="1:6">
+      <c r="A40" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B40" s="6">
-        <f>_xll.CVX.VALUE(B21,B11)</f>
-        <v>1.3085414715514723E-10</v>
-      </c>
-      <c r="F40" s="1" t="s">
+      <c r="B40" s="7">
+        <f>CVX.VALUE(B21,B11)</f>
+        <v>0</v>
+      </c>
+      <c r="F40" s="2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A41" s="3" t="s">
+    <row r="41" spans="1:6">
+      <c r="A41" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B41" s="6">
-        <f>_xll.CVX.VALUE(B21,B12)</f>
-        <v>4.0000000001052118</v>
-      </c>
-      <c r="F41" s="1" t="s">
+      <c r="B41" s="7">
+        <f>CVX.VALUE(B21,B12)</f>
+        <v>0</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A42" s="3" t="s">
+    <row r="42" spans="1:6">
+      <c r="A42" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B42" s="6" t="str">
-        <f>_xll.CVX.DESCRIBE(B21)</f>
-        <v>"diet_result" (cvx:result:815426d7-ae99-405e-a662-2016a93c6cd0): result: status=optimal, objective_value=7.200000000516517, variables=[2]</v>
-      </c>
-      <c r="F42" s="1" t="s">
+      <c r="B42" s="7">
+        <f>CVX.DESCRIBE(B21)</f>
+        <v>0</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A43" s="3" t="s">
+    <row r="43" spans="1:6">
+      <c r="A43" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B43" s="6" t="str">
-        <f>_xll.CVX.DESCRIBE(B15)</f>
-        <v>"calorie_requirement" (cvx:constr:78e573fa-df85-4eb6-8b14-a2015f106058): constraint: (120) * ("qty_bread") + (150) * ("qty_milk") &gt;= 600</v>
-      </c>
-      <c r="F43" s="1" t="s">
+      <c r="B43" s="7">
+        <f>CVX.DESCRIBE(B15)</f>
+        <v>0</v>
+      </c>
+      <c r="F43" s="2" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A44" s="3" t="s">
+    <row r="44" spans="1:6">
+      <c r="A44" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B44" s="6" t="str">
-        <f>_xll.CVX.DESCRIBE(B16)</f>
-        <v>"bread_nonneg" (cvx:constr:05d5830d-7b8a-41fa-817b-e850c3b05d70): constraint: "qty_bread" &gt;= 0</v>
-      </c>
-      <c r="F44" s="1" t="s">
+      <c r="B44" s="7">
+        <f>CVX.DESCRIBE(B16)</f>
+        <v>0</v>
+      </c>
+      <c r="F44" s="2" t="s">
         <v>73</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="B37:E37"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B37:E37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>